<commit_message>
actualiza seleccion final con portafolios
</commit_message>
<xml_diff>
--- a/datos/seleccion_final_complexity.xlsx
+++ b/datos/seleccion_final_complexity.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="intensivo" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="extensivo" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="extensivo_portafolios" sheetId="3" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="100">
   <si>
     <t xml:space="preserve">Clusters</t>
   </si>
@@ -309,6 +310,18 @@
   </si>
   <si>
     <t xml:space="preserve">Fabricación de cuerdas, cordeles, bramantes y redes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lhf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">todos</t>
   </si>
 </sst>
 </file>
@@ -323,6 +336,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -341,8 +355,8 @@
     </font>
     <font>
       <sz val="12"/>
-      <name val=""/>
-      <family val="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -388,12 +402,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -417,652 +435,652 @@
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52.39"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="81.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="81.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="132.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>2651</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>1629</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>1.02</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>3.78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="132.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>2930</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>1629</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>1.02</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="2" t="n">
         <v>3.78</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="116.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>2013</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>868</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>1.31</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="2" t="n">
         <v>2.93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="247.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>2100</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>2869</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>1.28</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="2" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>2391</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>112</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>1.15</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="G6" s="2" t="n">
         <v>-0.59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="69.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>2394</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>676</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>2.74</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="G7" s="2" t="n">
         <v>-1.19</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="243.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>2090</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>1.53</v>
       </c>
-      <c r="G8" s="1" t="n">
+      <c r="G8" s="2" t="n">
         <v>-1.25</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>1062</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>5.05</v>
       </c>
-      <c r="G9" s="1" t="n">
+      <c r="G9" s="2" t="n">
         <v>1.32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>1103</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>925</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>2.42</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="G10" s="2" t="n">
         <v>-0.31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>1050</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>4783</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>2.74</v>
       </c>
-      <c r="G11" s="1" t="n">
+      <c r="G11" s="2" t="n">
         <v>-0.63</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>1080</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>2036</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>3.47</v>
       </c>
-      <c r="G12" s="1" t="n">
+      <c r="G12" s="2" t="n">
         <v>-0.88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="139.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>1020</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>2923</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>3.46</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="2" t="n">
         <v>-1.11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="132.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>7320</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>1237</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>2.53</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="G14" s="2" t="n">
         <v>-0.37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="87.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>8220</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>3662</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>1.55</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G15" s="2" t="n">
         <v>-2.74</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="99.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>7990</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>962</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>3.38</v>
       </c>
-      <c r="G16" s="1" t="n">
+      <c r="G16" s="2" t="n">
         <v>1.45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="121.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>7721</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>178</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="2" t="n">
         <v>1.63</v>
       </c>
-      <c r="G17" s="1" t="n">
+      <c r="G17" s="2" t="n">
         <v>0.6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="87.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>5110</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>1009</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>1.47</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G18" s="2" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>5011</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>576</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>1.33</v>
       </c>
-      <c r="G19" s="1" t="n">
+      <c r="G19" s="2" t="n">
         <v>-0.2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="139.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>5222</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>1560</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>3.06</v>
       </c>
-      <c r="G20" s="1" t="n">
+      <c r="G20" s="2" t="n">
         <v>-0.54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>7710</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>795</v>
       </c>
-      <c r="F21" s="1" t="n">
+      <c r="F21" s="2" t="n">
         <v>1.08</v>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="G21" s="2" t="n">
         <v>-0.77</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>2030</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>857</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>7.39</v>
       </c>
-      <c r="G22" s="1" t="n">
+      <c r="G22" s="2" t="n">
         <v>1.1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="69.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>1313</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>71320</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>100.29</v>
       </c>
-      <c r="G23" s="1" t="n">
+      <c r="G23" s="2" t="n">
         <v>-1.28</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>1391</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>2839</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>26.87</v>
       </c>
-      <c r="G24" s="1" t="n">
+      <c r="G24" s="2" t="n">
         <v>-1.57</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="87.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>1311</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>9914</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>31.93</v>
       </c>
-      <c r="G25" s="1" t="n">
+      <c r="G25" s="2" t="n">
         <v>-2.14</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="104.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>1399</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>3752</v>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>6.3</v>
       </c>
-      <c r="G26" s="1" t="n">
+      <c r="G26" s="2" t="n">
         <v>-2.64</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="174.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>1392</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>9677</v>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>13.38</v>
       </c>
-      <c r="G27" s="1" t="n">
+      <c r="G27" s="2" t="n">
         <v>-3.06</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="121.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>1410</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>16142</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>4.69</v>
       </c>
-      <c r="G28" s="1" t="n">
+      <c r="G28" s="2" t="n">
         <v>-3.35</v>
       </c>
     </row>
@@ -1085,677 +1103,1717 @@
   <dimension ref="A1:G29"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="55.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="83.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="55.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="83.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="116.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>2910</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>1.49</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="F2" s="2" t="n">
         <v>6.96</v>
       </c>
-      <c r="G2" s="1" t="n">
+      <c r="G2" s="2" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>2816</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>1.92</v>
       </c>
-      <c r="F3" s="1" t="n">
+      <c r="F3" s="2" t="n">
         <v>6.85</v>
       </c>
-      <c r="G3" s="1" t="n">
+      <c r="G3" s="2" t="n">
         <v>0.16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>2829</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>1.92</v>
       </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>6.85</v>
       </c>
-      <c r="G4" s="1" t="n">
+      <c r="G4" s="2" t="n">
         <v>0.16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>3040</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>1.59</v>
       </c>
-      <c r="F5" s="1" t="n">
+      <c r="F5" s="2" t="n">
         <v>6.7</v>
       </c>
-      <c r="G5" s="1" t="n">
+      <c r="G5" s="2" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>2815</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>1.63</v>
       </c>
-      <c r="F6" s="1" t="n">
+      <c r="F6" s="2" t="n">
         <v>5.7</v>
       </c>
-      <c r="G6" s="1" t="n">
+      <c r="G6" s="2" t="n">
         <v>0.13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>2811</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>1.49</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="2" t="n">
         <v>5.32</v>
       </c>
-      <c r="G7" s="1" t="n">
+      <c r="G7" s="2" t="n">
         <v>0.13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>2819</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>1.44</v>
       </c>
-      <c r="F8" s="1" t="n">
+      <c r="F8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="1" t="n">
+      <c r="G8" s="2" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>2822</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>1.44</v>
       </c>
-      <c r="F9" s="1" t="n">
+      <c r="F9" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="1" t="n">
+      <c r="G9" s="2" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>2591</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>1.79</v>
       </c>
-      <c r="F10" s="1" t="n">
+      <c r="F10" s="2" t="n">
         <v>4.62</v>
       </c>
-      <c r="G10" s="1" t="n">
+      <c r="G10" s="2" t="n">
         <v>0.17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>2660</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>1.75</v>
       </c>
-      <c r="F11" s="1" t="n">
+      <c r="F11" s="2" t="n">
         <v>4.57</v>
       </c>
-      <c r="G11" s="1" t="n">
+      <c r="G11" s="2" t="n">
         <v>0.17</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>2420</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="F12" s="1" t="n">
+      <c r="F12" s="2" t="n">
         <v>0.84</v>
       </c>
-      <c r="G12" s="1" t="n">
+      <c r="G12" s="2" t="n">
         <v>0.27</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="99.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>2011</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>1.74</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <v>5.56</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="2" t="n">
         <v>0.18</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>2395</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>0.74</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <v>0.58</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="G14" s="2" t="n">
         <v>0.28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>2012</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>0.6</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <v>-0.02</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G15" s="2" t="n">
         <v>0.29</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>2021</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>0.34</v>
       </c>
-      <c r="F16" s="1" t="n">
+      <c r="F16" s="2" t="n">
         <v>-1.01</v>
       </c>
-      <c r="G16" s="1" t="n">
+      <c r="G16" s="2" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>1920</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>0.25</v>
       </c>
-      <c r="F17" s="1" t="n">
+      <c r="F17" s="2" t="n">
         <v>-1.68</v>
       </c>
-      <c r="G17" s="1" t="n">
+      <c r="G17" s="2" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>1075</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>1.33</v>
       </c>
-      <c r="F18" s="1" t="n">
+      <c r="F18" s="2" t="n">
         <v>4.15</v>
       </c>
-      <c r="G18" s="1" t="n">
+      <c r="G18" s="2" t="n">
         <v>0.22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>1061</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="F19" s="1" t="n">
+      <c r="F19" s="2" t="n">
         <v>-0.45</v>
       </c>
-      <c r="G19" s="1" t="n">
+      <c r="G19" s="2" t="n">
         <v>0.29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>1101</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>0.27</v>
       </c>
-      <c r="F20" s="1" t="n">
+      <c r="F20" s="2" t="n">
         <v>-1.45</v>
       </c>
-      <c r="G20" s="1" t="n">
+      <c r="G20" s="2" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>1073</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="1" t="n">
+      <c r="E21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="n">
         <v>-2.68</v>
       </c>
-      <c r="G21" s="1" t="n">
+      <c r="G21" s="2" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>7110</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>1.46</v>
       </c>
-      <c r="F22" s="1" t="n">
+      <c r="F22" s="2" t="n">
         <v>3.69</v>
       </c>
-      <c r="G22" s="1" t="n">
+      <c r="G22" s="2" t="n">
         <v>0.23</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>8291</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>1.42</v>
       </c>
-      <c r="F23" s="1" t="n">
+      <c r="F23" s="2" t="n">
         <v>3.45</v>
       </c>
-      <c r="G23" s="1" t="n">
+      <c r="G23" s="2" t="n">
         <v>0.22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>6910</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>1.31</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="2" t="n">
         <v>2.76</v>
       </c>
-      <c r="G24" s="1" t="n">
+      <c r="G24" s="2" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>7020</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>0.55</v>
       </c>
-      <c r="F25" s="1" t="n">
+      <c r="F25" s="2" t="n">
         <v>0.18</v>
       </c>
-      <c r="G25" s="1" t="n">
+      <c r="G25" s="2" t="n">
         <v>0.29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>5021</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>1.62</v>
       </c>
-      <c r="F26" s="1" t="n">
+      <c r="F26" s="2" t="n">
         <v>4.17</v>
       </c>
-      <c r="G26" s="1" t="n">
+      <c r="G26" s="2" t="n">
         <v>0.16</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>5224</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>0.61</v>
       </c>
-      <c r="F27" s="1" t="n">
+      <c r="F27" s="2" t="n">
         <v>0.45</v>
       </c>
-      <c r="G27" s="1" t="n">
+      <c r="G27" s="2" t="n">
         <v>0.28</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>7911</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E28" s="1" t="n">
+      <c r="E28" s="2" t="n">
         <v>0.22</v>
       </c>
-      <c r="F28" s="1" t="n">
+      <c r="F28" s="2" t="n">
         <v>-1.39</v>
       </c>
-      <c r="G28" s="1" t="n">
+      <c r="G28" s="2" t="n">
         <v>0.31</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="2" t="n">
         <v>1394</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E29" s="1" t="n">
+      <c r="E29" s="2" t="n">
         <v>0.45</v>
       </c>
-      <c r="F29" s="1" t="n">
+      <c r="F29" s="2" t="n">
         <v>-0.25</v>
       </c>
-      <c r="G29" s="1" t="n">
+      <c r="G29" s="2" t="n">
         <v>0.3</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="55.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="83.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46.13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2910</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2816</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2829</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3040</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2815</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2811</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2819</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2822</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2591</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H10" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2660</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>4.57</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2420</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="H12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="99.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>2395</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1920</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>-1.68</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>1075</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H18" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>1101</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>-1.45</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1073</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>-2.68</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="H21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>7110</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>8291</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="H23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>6910</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>7020</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>5021</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>5224</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7911</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>-1.39</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="H28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>1394</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>